<commit_message>
Geology system finally done
</commit_message>
<xml_diff>
--- a/resources/Лист Microsoft Excel.xlsx
+++ b/resources/Лист Microsoft Excel.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C96B493-4249-44E2-8CB9-8B8912ED8299}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3655305-A7E5-495C-B6C7-1453D3FFC6E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="183">
   <si>
     <t>Название</t>
   </si>
@@ -565,13 +565,10 @@
     <t>Structure</t>
   </si>
   <si>
-    <t>Processor</t>
-  </si>
-  <si>
-    <t>Color</t>
-  </si>
-  <si>
     <t>d</t>
+  </si>
+  <si>
+    <t>Feature</t>
   </si>
 </sst>
 </file>
@@ -588,24 +585,17 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -622,7 +612,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -903,7 +893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E128"/>
+  <dimension ref="A1:D128"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -916,7 +906,7 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -927,13 +917,10 @@
         <v>180</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>108</v>
       </c>
@@ -944,10 +931,10 @@
         <v>176</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>98</v>
       </c>
@@ -958,10 +945,10 @@
         <v>177</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>40</v>
       </c>
@@ -972,10 +959,10 @@
         <v>172</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>137</v>
       </c>
@@ -986,10 +973,10 @@
         <v>174</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>138</v>
       </c>
@@ -1000,10 +987,10 @@
         <v>179</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>69</v>
       </c>
@@ -1014,10 +1001,10 @@
         <v>174</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
@@ -1028,7 +1015,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>76</v>
       </c>
@@ -1039,7 +1026,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>74</v>
       </c>
@@ -1050,7 +1037,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -1061,7 +1048,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>82</v>
       </c>
@@ -1072,7 +1059,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>9</v>
       </c>
@@ -1083,7 +1070,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>57</v>
       </c>
@@ -1094,7 +1081,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
@@ -1105,7 +1092,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>122</v>
       </c>
@@ -2349,9 +2336,10 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:C128">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C128">
     <sortCondition ref="A2"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>